<commit_message>
v2: working paper (chapter form) and journal article (IMRAD) with review matrix, data appendix, new CLAUDE.md and README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BJh4xwEjPS1QoGpFfUAH88
</commit_message>
<xml_diff>
--- a/codebook/codebook.xlsx
+++ b/codebook/codebook.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,27 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Raw, S12: Published coefficients of the reference study (Annex Tables 1-2, Figure 7)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>as published</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1214,7 +1235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D149"/>
+  <dimension ref="A1:D160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -4496,6 +4517,248 @@
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>outcome</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>shock</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>se</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>signif</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>obs</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>n_units</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>as published by the source</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>data/reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>adj_r2</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
         <is>
           <t>as published by the source</t>
         </is>
@@ -12395,7 +12658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -12975,6 +13238,53 @@
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Kpodar and Liu (2021), IMF Working Paper WP/21/271</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Published coefficients of the reference study (Annex Tables 1-2, Figure 7)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Comparison of the Philippine pass-through with the reference study's estimates</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>reference/kpodar_liu_2021_targets.csv</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.imf.org/en/publications/wp/issues/2021/11/12/the-distributional-implications-of-the-impact-of-fuel-price-increases-on-inflation-506822</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Advanced and developing economies, 2000-2019</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Typed from the published paper</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>

</xml_diff>